<commit_message>
adding sample sheet functionality
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,13 +8,21 @@
   </bookViews>
   <sheets>
     <sheet name="Digestion" sheetId="1" r:id="rId1"/>
+    <sheet name="200126512" sheetId="2" r:id="rId2"/>
+    <sheet name="200126511" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+  <si>
+    <t>Date:</t>
+  </si>
+  <si>
+    <t>Request ID:</t>
+  </si>
   <si>
     <t>Microwave</t>
   </si>
@@ -70,29 +78,53 @@
     <t>200127586_2</t>
   </si>
   <si>
-    <t>Katanax</t>
-  </si>
-  <si>
-    <t>Ti, Si</t>
-  </si>
-  <si>
-    <t>200127587_1</t>
-  </si>
-  <si>
-    <t>200127587_2</t>
-  </si>
-  <si>
-    <t>Hotplate</t>
-  </si>
-  <si>
-    <t>Ag, Pd</t>
+    <t>sample</t>
+  </si>
+  <si>
+    <t>Dilution</t>
+  </si>
+  <si>
+    <t>conc. [mg/L]</t>
+  </si>
+  <si>
+    <t>Ni_ppm</t>
+  </si>
+  <si>
+    <t>%Ni</t>
+  </si>
+  <si>
+    <t>200126511_1</t>
+  </si>
+  <si>
+    <t>200126511_2</t>
+  </si>
+  <si>
+    <t>200126512_1</t>
+  </si>
+  <si>
+    <t>200126512_2</t>
+  </si>
+  <si>
+    <t>Ti_ppm</t>
+  </si>
+  <si>
+    <t>%Ti</t>
+  </si>
+  <si>
+    <t>200126513_1</t>
+  </si>
+  <si>
+    <t>200126513_2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,6 +134,15 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -144,13 +185,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,11 +491,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -457,43 +502,21 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2">
+        <v>46132</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2">
+        <v>100482511</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -501,228 +524,274 @@
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="2" t="s">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="E12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="3"/>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
+  <mergeCells count="7">
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B7:E7"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="I2:J2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="9:10">
+      <c r="I2">
+        <f>Digestion!B17</f>
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <f>Digestion!C17</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
not much done at work
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -658,15 +658,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="I2:J2"/>
+  <dimension ref="G2:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="9:10">
-      <c r="I2">
+    <row r="2" spans="7:8">
+      <c r="G2">
         <f>Digestion!B17</f>
         <v>0</v>
       </c>
-      <c r="J2">
+      <c r="H2">
         <f>Digestion!C17</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
need to fix the issues of some not showing from the gui
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,15 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Digestion" sheetId="1" r:id="rId1"/>
-    <sheet name="200126512" sheetId="2" r:id="rId2"/>
-    <sheet name="200126511" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>Date:</t>
   </si>
@@ -78,43 +76,31 @@
     <t>200127586_2</t>
   </si>
   <si>
-    <t>sample</t>
-  </si>
-  <si>
-    <t>Dilution</t>
-  </si>
-  <si>
-    <t>conc. [mg/L]</t>
-  </si>
-  <si>
-    <t>Ni_ppm</t>
-  </si>
-  <si>
-    <t>%Ni</t>
-  </si>
-  <si>
-    <t>200126511_1</t>
-  </si>
-  <si>
-    <t>200126511_2</t>
-  </si>
-  <si>
-    <t>200126512_1</t>
-  </si>
-  <si>
-    <t>200126512_2</t>
-  </si>
-  <si>
-    <t>Ti_ppm</t>
-  </si>
-  <si>
-    <t>%Ti</t>
-  </si>
-  <si>
-    <t>200126513_1</t>
-  </si>
-  <si>
-    <t>200126513_2</t>
+    <t>200127586_3</t>
+  </si>
+  <si>
+    <t>200127587_1</t>
+  </si>
+  <si>
+    <t>200127587_2</t>
+  </si>
+  <si>
+    <t>200127587_3</t>
+  </si>
+  <si>
+    <t>Katanax</t>
+  </si>
+  <si>
+    <t>Ti, Si</t>
+  </si>
+  <si>
+    <t>200127588_1</t>
+  </si>
+  <si>
+    <t>200127588_2</t>
+  </si>
+  <si>
+    <t>200127588_3</t>
   </si>
 </sst>
 </file>
@@ -124,7 +110,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,15 +120,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -185,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -196,7 +173,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,10 +467,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -503,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46132</v>
+        <v>46133</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -642,8 +619,131 @@
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
     </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="5"/>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="11">
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B7:E7"/>
@@ -651,147 +751,11 @@
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B11:E11"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="G2:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="2" spans="7:8">
-      <c r="G2">
-        <f>Digestion!B17</f>
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <f>Digestion!C17</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
wrote cleaner code that don't requrie looking intoDigestion.element_list
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,13 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Digestion" sheetId="1" r:id="rId1"/>
+    <sheet name="200127586" sheetId="2" r:id="rId2"/>
+    <sheet name="200127587" sheetId="3" r:id="rId3"/>
+    <sheet name="200127588" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="40">
   <si>
     <t>Date:</t>
   </si>
@@ -101,6 +104,39 @@
   </si>
   <si>
     <t>200127588_3</t>
+  </si>
+  <si>
+    <t>sample</t>
+  </si>
+  <si>
+    <t>Dilution</t>
+  </si>
+  <si>
+    <t>conc. [mg/L]</t>
+  </si>
+  <si>
+    <t>Ca_ppm</t>
+  </si>
+  <si>
+    <t>%Ca</t>
+  </si>
+  <si>
+    <t>Cu_ppm</t>
+  </si>
+  <si>
+    <t>%Cu</t>
+  </si>
+  <si>
+    <t>Ti_ppm</t>
+  </si>
+  <si>
+    <t>%Ti</t>
+  </si>
+  <si>
+    <t>Si_ppm</t>
+  </si>
+  <si>
+    <t>%Si</t>
   </si>
 </sst>
 </file>
@@ -110,7 +146,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,6 +156,15 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -162,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -173,6 +218,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,4 +804,710 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>100482511</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="G6">
+        <f>Digestion!B17</f>
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <f>Digestion!C17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="G7">
+        <f>Digestion!B18</f>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f>Digestion!C18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="G8">
+        <f>Digestion!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <f>Digestion!C19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="G12">
+        <f>Digestion!B17</f>
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <f>Digestion!C17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="G13">
+        <f>Digestion!B18</f>
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <f>Digestion!C18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="G14">
+        <f>Digestion!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <f>Digestion!C19</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>100482511</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="G6">
+        <f>Digestion!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <f>Digestion!C20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="G7">
+        <f>Digestion!B21</f>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f>Digestion!C21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="G8">
+        <f>Digestion!B22</f>
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <f>Digestion!C22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="G12">
+        <f>Digestion!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <f>Digestion!C20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="G13">
+        <f>Digestion!B21</f>
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <f>Digestion!C21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="G14">
+        <f>Digestion!B22</f>
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <f>Digestion!C22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="G18">
+        <f>Digestion!B30</f>
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <f>Digestion!C30</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="G19">
+        <f>Digestion!B31</f>
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <f>Digestion!C31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="G20">
+        <f>Digestion!B32</f>
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <f>Digestion!C32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="G24">
+        <f>Digestion!B30</f>
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <f>Digestion!C30</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="G25">
+        <f>Digestion!B31</f>
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <f>Digestion!C31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="G26">
+        <f>Digestion!B32</f>
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <f>Digestion!C32</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>100482511</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="G6">
+        <f>Digestion!B33</f>
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <f>Digestion!C33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="G7">
+        <f>Digestion!B34</f>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f>Digestion!C34</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="G8">
+        <f>Digestion!B35</f>
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <f>Digestion!C35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="G12">
+        <f>Digestion!B33</f>
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <f>Digestion!C33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="G13">
+        <f>Digestion!B34</f>
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <f>Digestion!C34</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="G14">
+        <f>Digestion!B35</f>
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <f>Digestion!C35</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added most functionality, except for titration
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="43">
   <si>
     <t>Date:</t>
   </si>
@@ -119,6 +119,15 @@
   </si>
   <si>
     <t>%Ca</t>
+  </si>
+  <si>
+    <t>reported result:</t>
+  </si>
+  <si>
+    <t>oxide factor:</t>
+  </si>
+  <si>
+    <t>lot:</t>
   </si>
   <si>
     <t>Cu_ppm</t>
@@ -143,9 +152,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00&quot; ppm&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot; %&quot;"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -208,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -221,6 +232,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,7 +551,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46134</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -810,7 +833,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -822,7 +845,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46134</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -860,7 +883,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="7">
-        <f>((C6)*(H6)*(I6))/(G6)</f>
+        <f>((C6)*(H6)*(I6))/(G6*1)</f>
         <v>0</v>
       </c>
       <c r="E6" s="7">
@@ -890,7 +913,7 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="7">
-        <f>((C7)*(H7)*(I7))/(G7)</f>
+        <f>((C7)*(H7)*(I7))/(G7*1)</f>
         <v>0</v>
       </c>
       <c r="E7" s="7">
@@ -920,7 +943,7 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="7">
-        <f>((C8)*(H8)*(I8))/(G8)</f>
+        <f>((C8)*(H8)*(I8))/(G8*1)</f>
         <v>0</v>
       </c>
       <c r="E8" s="7">
@@ -940,121 +963,227 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="9">
+        <f>AVERAGE(D6:D8)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="8"/>
+      <c r="C11" s="10">
+        <f>AVERAGE(E6:E8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="11"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="10">
+        <f>AVERAGE(E6:E8)*(C12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="6" t="s">
+      <c r="D16" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="7">
+        <f>((C17)*(H17)*(I17))/(G17*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="7">
+        <f>D17/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <f>Digestion!B17</f>
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <f>Digestion!C17</f>
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <f>(LEFT(B17,FIND("/",B17)-1)/RIGHT(B17,LEN(B17)-FIND("/", B17)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="7">
+        <f>((C18)*(H18)*(I18))/(G18*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="7">
+        <f>D18/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <f>Digestion!B18</f>
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <f>Digestion!C18</f>
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <f>(LEFT(B18,FIND("/",B18)-1)/RIGHT(B18,LEN(B18)-FIND("/", B18)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="7">
+        <f>((C19)*(H19)*(I19))/(G19*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="7">
+        <f>D19/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <f>Digestion!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <f>Digestion!C19</f>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <f>(LEFT(B19,FIND("/",B19)-1)/RIGHT(B19,LEN(B19)-FIND("/", B19)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9">
+        <f>AVERAGE(D17:D19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="10">
+        <f>AVERAGE(E17:E19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="8" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="7">
-        <f>((C12)*(H12)*(I12))/(G12)</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="7">
-        <f>D12/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <f>Digestion!B17</f>
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <f>Digestion!C17</f>
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <f>(LEFT(B12,FIND("/",B12)-1)/RIGHT(B12,LEN(B12)-FIND("/", B12)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="7">
-        <f>((C13)*(H13)*(I13))/(G13)</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="7">
-        <f>D13/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <f>Digestion!B18</f>
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <f>Digestion!C18</f>
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <f>(LEFT(B13,FIND("/",B13)-1)/RIGHT(B13,LEN(B13)-FIND("/", B13)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="7">
-        <f>((C14)*(H14)*(I14))/(G14)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="7">
-        <f>D14/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <f>Digestion!B19</f>
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <f>Digestion!C19</f>
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <f>(LEFT(B14,FIND("/",B14)-1)/RIGHT(B14,LEN(B14)-FIND("/", B14)))</f>
-        <v>0</v>
-      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="11"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8"/>
+      <c r="C24" s="10">
+        <f>AVERAGE(E17:E19)*(C23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="8"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
     </row>
   </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:E25"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -1066,7 +1195,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46134</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1104,7 +1233,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="7">
-        <f>((C6)*(H6)*(I6))/(G6)</f>
+        <f>((C6)*(H6)*(I6))/(G6*1)</f>
         <v>0</v>
       </c>
       <c r="E6" s="7">
@@ -1134,7 +1263,7 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="7">
-        <f>((C7)*(H7)*(I7))/(G7)</f>
+        <f>((C7)*(H7)*(I7))/(G7*1)</f>
         <v>0</v>
       </c>
       <c r="E7" s="7">
@@ -1164,7 +1293,7 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="7">
-        <f>((C8)*(H8)*(I8))/(G8)</f>
+        <f>((C8)*(H8)*(I8))/(G8*1)</f>
         <v>0</v>
       </c>
       <c r="E8" s="7">
@@ -1184,133 +1313,102 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="9">
+        <f>AVERAGE(D6:D8)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="8"/>
+      <c r="C11" s="10">
+        <f>AVERAGE(E6:E8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="11"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="10">
+        <f>AVERAGE(E6:E8)*(C12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="7">
-        <f>((C12)*(H12)*(I12))/(G12)</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="7">
-        <f>D12/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <f>Digestion!B20</f>
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <f>Digestion!C20</f>
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <f>(LEFT(B12,FIND("/",B12)-1)/RIGHT(B12,LEN(B12)-FIND("/", B12)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="7">
-        <f>((C13)*(H13)*(I13))/(G13)</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="7">
-        <f>D13/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <f>Digestion!B21</f>
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <f>Digestion!C21</f>
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <f>(LEFT(B13,FIND("/",B13)-1)/RIGHT(B13,LEN(B13)-FIND("/", B13)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="7">
-        <f>((C14)*(H14)*(I14))/(G14)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="7">
-        <f>D14/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <f>Digestion!B22</f>
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <f>Digestion!C22</f>
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <f>(LEFT(B14,FIND("/",B14)-1)/RIGHT(B14,LEN(B14)-FIND("/", B14)))</f>
-        <v>0</v>
+      <c r="D16" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>37</v>
+        <v>21</v>
+      </c>
+      <c r="B17" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="7">
+        <f>((C17)*(H17)*(I17))/(G17*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="7">
+        <f>D17/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <f>Digestion!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <f>Digestion!C20</f>
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <f>(LEFT(B17,FIND("/",B17)-1)/RIGHT(B17,LEN(B17)-FIND("/", B17)))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B18" s="5">
         <f>"1/1"</f>
@@ -1318,7 +1416,7 @@
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="7">
-        <f>((C18)*(H18)*(I18))/(G18)</f>
+        <f>((C18)*(H18)*(I18))/(G18*1)</f>
         <v>0</v>
       </c>
       <c r="E18" s="7">
@@ -1326,11 +1424,11 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <f>Digestion!B30</f>
+        <f>Digestion!B21</f>
         <v>0</v>
       </c>
       <c r="H18">
-        <f>Digestion!C30</f>
+        <f>Digestion!C21</f>
         <v>0</v>
       </c>
       <c r="I18">
@@ -1340,7 +1438,7 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B19" s="5">
         <f>"1/1"</f>
@@ -1348,7 +1446,7 @@
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="7">
-        <f>((C19)*(H19)*(I19))/(G19)</f>
+        <f>((C19)*(H19)*(I19))/(G19*1)</f>
         <v>0</v>
       </c>
       <c r="E19" s="7">
@@ -1356,11 +1454,11 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <f>Digestion!B31</f>
+        <f>Digestion!B22</f>
         <v>0</v>
       </c>
       <c r="H19">
-        <f>Digestion!C31</f>
+        <f>Digestion!C22</f>
         <v>0</v>
       </c>
       <c r="I19">
@@ -1368,151 +1466,392 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="4" t="s">
+    <row r="21" spans="1:9">
+      <c r="A21" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9">
+        <f>AVERAGE(D17:D19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="10">
+        <f>AVERAGE(E17:E19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="11"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8"/>
+      <c r="C24" s="10">
+        <f>AVERAGE(E17:E19)*(C23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="8"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="7">
+        <f>((C28)*(H28)*(I28))/(G28*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="7">
+        <f>D28/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <f>Digestion!B30</f>
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <f>Digestion!C30</f>
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <f>(LEFT(B28,FIND("/",B28)-1)/RIGHT(B28,LEN(B28)-FIND("/", B28)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="7">
+        <f>((C29)*(H29)*(I29))/(G29*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="7">
+        <f>D29/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <f>Digestion!B31</f>
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <f>Digestion!C31</f>
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <f>(LEFT(B29,FIND("/",B29)-1)/RIGHT(B29,LEN(B29)-FIND("/", B29)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="7">
-        <f>((C20)*(H20)*(I20))/(G20)</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="7">
-        <f>D20/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G20">
+      <c r="B30" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="7">
+        <f>((C30)*(H30)*(I30))/(G30*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="7">
+        <f>D30/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G30">
         <f>Digestion!B32</f>
         <v>0</v>
       </c>
-      <c r="H20">
+      <c r="H30">
         <f>Digestion!C32</f>
         <v>0</v>
       </c>
-      <c r="I20">
-        <f>(LEFT(B20,FIND("/",B20)-1)/RIGHT(B20,LEN(B20)-FIND("/", B20)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="4" t="s">
+      <c r="I30">
+        <f>(LEFT(B30,FIND("/",B30)-1)/RIGHT(B30,LEN(B30)-FIND("/", B30)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="8"/>
+      <c r="C32" s="9">
+        <f>AVERAGE(D28:D30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="8"/>
+      <c r="C33" s="10">
+        <f>AVERAGE(E28:E30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="8"/>
+      <c r="C34" s="11"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="8"/>
+      <c r="C35" s="10">
+        <f>AVERAGE(E28:E30)*(C34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="8"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C38" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="4" t="s">
+      <c r="D38" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="7">
-        <f>((C24)*(H24)*(I24))/(G24)</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="7">
-        <f>D24/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G24">
+      <c r="B39" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="5"/>
+      <c r="D39" s="7">
+        <f>((C39)*(H39)*(I39))/(G39*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="7">
+        <f>D39/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G39">
         <f>Digestion!B30</f>
         <v>0</v>
       </c>
-      <c r="H24">
+      <c r="H39">
         <f>Digestion!C30</f>
         <v>0</v>
       </c>
-      <c r="I24">
-        <f>(LEFT(B24,FIND("/",B24)-1)/RIGHT(B24,LEN(B24)-FIND("/", B24)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="4" t="s">
+      <c r="I39">
+        <f>(LEFT(B39,FIND("/",B39)-1)/RIGHT(B39,LEN(B39)-FIND("/", B39)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="7">
-        <f>((C25)*(H25)*(I25))/(G25)</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="7">
-        <f>D25/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G25">
+      <c r="B40" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="7">
+        <f>((C40)*(H40)*(I40))/(G40*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="7">
+        <f>D40/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G40">
         <f>Digestion!B31</f>
         <v>0</v>
       </c>
-      <c r="H25">
+      <c r="H40">
         <f>Digestion!C31</f>
         <v>0</v>
       </c>
-      <c r="I25">
-        <f>(LEFT(B25,FIND("/",B25)-1)/RIGHT(B25,LEN(B25)-FIND("/", B25)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="4" t="s">
+      <c r="I40">
+        <f>(LEFT(B40,FIND("/",B40)-1)/RIGHT(B40,LEN(B40)-FIND("/", B40)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="7">
-        <f>((C26)*(H26)*(I26))/(G26)</f>
-        <v>0</v>
-      </c>
-      <c r="E26" s="7">
-        <f>D26/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G26">
+      <c r="B41" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="5"/>
+      <c r="D41" s="7">
+        <f>((C41)*(H41)*(I41))/(G41*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="7">
+        <f>D41/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G41">
         <f>Digestion!B32</f>
         <v>0</v>
       </c>
-      <c r="H26">
+      <c r="H41">
         <f>Digestion!C32</f>
         <v>0</v>
       </c>
-      <c r="I26">
-        <f>(LEFT(B26,FIND("/",B26)-1)/RIGHT(B26,LEN(B26)-FIND("/", B26)))</f>
-        <v>0</v>
-      </c>
+      <c r="I41">
+        <f>(LEFT(B41,FIND("/",B41)-1)/RIGHT(B41,LEN(B41)-FIND("/", B41)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" s="8"/>
+      <c r="C43" s="9">
+        <f>AVERAGE(D39:D41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B44" s="8"/>
+      <c r="C44" s="10">
+        <f>AVERAGE(E39:E41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B45" s="8"/>
+      <c r="C45" s="11"/>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46" s="8"/>
+      <c r="C46" s="10">
+        <f>AVERAGE(E39:E41)*(C45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B47" s="8"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
     </row>
   </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:E47"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -1524,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46134</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1546,10 +1885,10 @@
         <v>31</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1562,7 +1901,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="7">
-        <f>((C6)*(H6)*(I6))/(G6)</f>
+        <f>((C6)*(H6)*(I6))/(G6*1)</f>
         <v>0</v>
       </c>
       <c r="E6" s="7">
@@ -1592,7 +1931,7 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="7">
-        <f>((C7)*(H7)*(I7))/(G7)</f>
+        <f>((C7)*(H7)*(I7))/(G7*1)</f>
         <v>0</v>
       </c>
       <c r="E7" s="7">
@@ -1622,7 +1961,7 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="7">
-        <f>((C8)*(H8)*(I8))/(G8)</f>
+        <f>((C8)*(H8)*(I8))/(G8*1)</f>
         <v>0</v>
       </c>
       <c r="E8" s="7">
@@ -1642,114 +1981,220 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="9">
+        <f>AVERAGE(D6:D8)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="8"/>
+      <c r="C11" s="10">
+        <f>AVERAGE(E6:E8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="11"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="10">
+        <f>AVERAGE(E6:E8)*(C12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="4" t="s">
+      <c r="D16" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="7">
-        <f>((C12)*(H12)*(I12))/(G12)</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="7">
-        <f>D12/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G12">
+      <c r="B17" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="7">
+        <f>((C17)*(H17)*(I17))/(G17*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="7">
+        <f>D17/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G17">
         <f>Digestion!B33</f>
         <v>0</v>
       </c>
-      <c r="H12">
+      <c r="H17">
         <f>Digestion!C33</f>
         <v>0</v>
       </c>
-      <c r="I12">
-        <f>(LEFT(B12,FIND("/",B12)-1)/RIGHT(B12,LEN(B12)-FIND("/", B12)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="4" t="s">
+      <c r="I17">
+        <f>(LEFT(B17,FIND("/",B17)-1)/RIGHT(B17,LEN(B17)-FIND("/", B17)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="7">
-        <f>((C13)*(H13)*(I13))/(G13)</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="7">
-        <f>D13/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G13">
+      <c r="B18" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="7">
+        <f>((C18)*(H18)*(I18))/(G18*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="7">
+        <f>D18/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G18">
         <f>Digestion!B34</f>
         <v>0</v>
       </c>
-      <c r="H13">
+      <c r="H18">
         <f>Digestion!C34</f>
         <v>0</v>
       </c>
-      <c r="I13">
-        <f>(LEFT(B13,FIND("/",B13)-1)/RIGHT(B13,LEN(B13)-FIND("/", B13)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="4" t="s">
+      <c r="I18">
+        <f>(LEFT(B18,FIND("/",B18)-1)/RIGHT(B18,LEN(B18)-FIND("/", B18)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="5">
-        <f>"1/1"</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="7">
-        <f>((C14)*(H14)*(I14))/(G14)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="7">
-        <f>D14/10000</f>
-        <v>0</v>
-      </c>
-      <c r="G14">
+      <c r="B19" s="5">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="7">
+        <f>((C19)*(H19)*(I19))/(G19*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="7">
+        <f>D19/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G19">
         <f>Digestion!B35</f>
         <v>0</v>
       </c>
-      <c r="H14">
+      <c r="H19">
         <f>Digestion!C35</f>
         <v>0</v>
       </c>
-      <c r="I14">
-        <f>(LEFT(B14,FIND("/",B14)-1)/RIGHT(B14,LEN(B14)-FIND("/", B14)))</f>
-        <v>0</v>
-      </c>
+      <c r="I19">
+        <f>(LEFT(B19,FIND("/",B19)-1)/RIGHT(B19,LEN(B19)-FIND("/", B19)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9">
+        <f>AVERAGE(D17:D19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="10">
+        <f>AVERAGE(E17:E19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="11"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="8"/>
+      <c r="C24" s="10">
+        <f>AVERAGE(E17:E19)*(C23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="8"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
     </row>
   </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:E25"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>